<commit_message>
Score sur 100% + dashboard mobile responsive + design modernisé
</commit_message>
<xml_diff>
--- a/resultats_participation.xlsx
+++ b/resultats_participation.xlsx
@@ -424,7 +424,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -472,7 +472,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Total (/90)</t>
+          <t>Total (/100)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 2/8 × 30 pts = 7.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 44.76% → 60.0% (+15.2 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 2/8 × 30 pts = 7.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 49.74% → 60.0% (+10.3 pts)</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 14+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 89.53% → 89.55% (+0.0 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 14+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 21+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 9 fork(s), R, documenté (+5) → 25/30 | Ajustement: 89.53% → 89.55% (+0.0 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 21+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 9 fork(s), R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 6/8 × 30 pts = 22.5/30 | GitHub: Dépôt trouvé (+5) | 15+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 82.46% → 80.0% (-2.5 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 6/8 × 30 pts = 22.5/30 | GitHub: Dépôt trouvé (+5) | 15+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 91.62% → 80.0% (-11.6 pts)</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 13+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 89.53% → 89.55% (+0.0 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 13+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tests: 5 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 4+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | documenté (+5) → 25/30 | Ajustement: 89.53% → 89.5% (-0.0 pts)</t>
+          <t>Tests: 5 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 4+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | documenté (+5) → 25/30 | Ajustement: 99.48% → 89.5% (-10.0 pts)</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Tests: 1 testé(s) × 20 pts = 20/40 | Présence: 8/8 × 30 pts = 30.0/30 | Profil GitHub: 2 repo(s) public(s) → 19/30 (format 15 + 4 bonus) | Ajustement: 65.03% → 79.0% (+14.0 pts)</t>
+          <t>Tests: 1 testé(s) × 20 pts = 20/40 | Présence: 8/8 × 30 pts = 30.0/30 | Profil GitHub: 2 repo(s) public(s) → 19/30 (format 15 + 4 bonus) | Ajustement: 72.25% → 79.0% (+6.8 pts)</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 19+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 1 star(s), R, documenté (+5) → 25/30 | Ajustement: 89.53% → 86.5% (-3.0 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 19+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 1 star(s), R, documenté (+5) → 25/30 | Ajustement: 99.48% → 86.5% (-13.0 pts)</t>
         </is>
       </c>
     </row>
@@ -860,11 +860,11 @@
         <v>25</v>
       </c>
       <c r="I10" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 2/8 × 30 pts = 7.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 44.76% → 52.0% (+7.2 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 2/8 × 30 pts = 7.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 49.74% → 52.0% (+2.3 pts)</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Tests: 4 testé(s) × 20 pts = 40/40 | Présence: 4/8 × 30 pts = 15.0/30 | GitHub: Dépôt trouvé (+5) | 2+ commit(s) (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 20/30 | Ajustement: 70.68% → 76.12% (+5.4 pts)</t>
+          <t>Tests: 4 testé(s) × 20 pts = 40/40 | Présence: 4/8 × 30 pts = 15.0/30 | GitHub: Dépôt trouvé (+5) | 2+ commit(s) (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 20/30 | Ajustement: 78.53% → 76.12% (-2.4 pts)</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 5/8 × 30 pts = 18.75/30 | GitHub: Dépôt trouvé (+5) | 12+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 78.93% → 79.48% (+0.5 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 5/8 × 30 pts = 18.75/30 | GitHub: Dépôt trouvé (+5) | 12+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 87.7% → 79.48% (-8.2 pts)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SIKATI 90%, Dupont/Arthur/Gamani 89.55%, reste intact
</commit_message>
<xml_diff>
--- a/resultats_participation.xlsx
+++ b/resultats_participation.xlsx
@@ -731,16 +731,16 @@
         <v>25</v>
       </c>
       <c r="I7" t="n">
-        <v>89.5</v>
+        <v>89.55</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>89.5%</t>
+          <t>89.55%</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tests: 5 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 4+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | documenté (+5) → 25/30 | Ajustement: 99.48% → 89.5% (-10.0 pts)</t>
+          <t>Tests: 5 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 4+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
         </is>
       </c>
     </row>
@@ -817,16 +817,16 @@
         <v>25</v>
       </c>
       <c r="I9" t="n">
-        <v>86.5</v>
+        <v>89.55</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>86.5%</t>
+          <t>89.55%</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 19+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 1 star(s), R, documenté (+5) → 25/30 | Ajustement: 99.48% → 86.5% (-13.0 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 19+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 1 star(s), R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
         </is>
       </c>
     </row>
@@ -860,16 +860,16 @@
         <v>25</v>
       </c>
       <c r="I10" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>90.0%</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Tests: 5 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 21+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 9 fork(s), R, documenté (+5) → 25/30</t>
+          <t>Tests: 5 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 21+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 9 fork(s), R, documenté (+5) → 25/30 | Ajustement: 100.0% → 90.0% (-10.0 pts)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Richelle 89.0%, Charonne 89.5%, Gamani/Dupont/Arthur 89.55%
</commit_message>
<xml_diff>
--- a/resultats_participation.xlsx
+++ b/resultats_participation.xlsx
@@ -602,16 +602,16 @@
         <v>25</v>
       </c>
       <c r="I4" t="n">
-        <v>89.55</v>
+        <v>89.5</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>89.55%</t>
+          <t>89.5%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 21+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 9 fork(s), R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 21+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | 9 fork(s), R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.5% (-10.0 pts)</t>
         </is>
       </c>
     </row>
@@ -688,16 +688,16 @@
         <v>25</v>
       </c>
       <c r="I6" t="n">
-        <v>89.55</v>
+        <v>89</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>89.55%</t>
+          <t>89.0%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 13+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.55% (-9.9 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub: Dépôt trouvé (+5) | 13+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 99.48% → 89.0% (-10.5 pts)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour scores: Biko 86.6%, Ismael/Girelle 85%, Anderson 83%, Rony 80%, Ivan 65% + nouveau membre TARH-YENGUE YANNICK 55%
</commit_message>
<xml_diff>
--- a/resultats_participation.xlsx
+++ b/resultats_participation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Résultats" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résultats" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -503,29 +503,29 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>6/8</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>40</v>
       </c>
       <c r="G2" t="n">
-        <v>7.5</v>
+        <v>22.5</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 2/8 × 30 pts = 7.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 49.74% → 60.0% (+10.3 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 6/8 × 30 pts = 22.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 65.45% → 80.0% (+14.5 pts)</t>
         </is>
       </c>
     </row>
@@ -632,29 +632,29 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6/8</t>
+          <t>7/8</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>22.5</v>
+        <v>26.25</v>
       </c>
       <c r="H5" t="n">
         <v>25</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>86.6%</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 6/8 × 30 pts = 22.5/30 | GitHub: Dépôt trouvé (+5) | 15+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 91.62% → 80.0% (-11.6 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 7/8 × 30 pts = 26.25/30 | GitHub: Dépôt trouvé (+5) | 15+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 95.55% → 86.6% (-9.0 pts)</t>
         </is>
       </c>
     </row>
@@ -771,19 +771,19 @@
         <v>30</v>
       </c>
       <c r="H8" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>79.0%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Tests: 1 testé(s) × 20 pts = 20/40 | Présence: 8/8 × 30 pts = 30.0/30 | Profil GitHub: 2 repo(s) public(s) → 19/30 (format 15 + 4 bonus) | Ajustement: 72.25% → 79.0% (+6.8 pts)</t>
+          <t>Tests: 1 testé(s) × 20 pts = 20/40 | Présence: 8/8 × 30 pts = 30.0/30 | GitHub ajusté: 25/30 | Ajustement: 78.53% → 85.0% (+6.5 pts)</t>
         </is>
       </c>
     </row>
@@ -890,29 +890,29 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>40</v>
       </c>
       <c r="G11" t="n">
-        <v>7.5</v>
+        <v>18.75</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 2/8 × 30 pts = 7.5/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 49.74% → 52.0% (+2.3 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 5/8 × 30 pts = 18.75/30 | Le lien fourni ne pointe pas vers GitHub. | Ajustement: 61.52% → 65.0% (+3.5 pts)</t>
         </is>
       </c>
     </row>
@@ -933,36 +933,36 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4/8</t>
+          <t>6/8</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>40</v>
       </c>
       <c r="G12" t="n">
-        <v>15</v>
+        <v>22.5</v>
       </c>
       <c r="H12" t="n">
         <v>20</v>
       </c>
       <c r="I12" t="n">
-        <v>76.12</v>
+        <v>83</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>76.12%</t>
+          <t>83.0%</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Tests: 4 testé(s) × 20 pts = 40/40 | Présence: 4/8 × 30 pts = 15.0/30 | GitHub: Dépôt trouvé (+5) | 2+ commit(s) (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 20/30 | Ajustement: 78.53% → 76.12% (-2.4 pts)</t>
+          <t>Tests: 4 testé(s) × 20 pts = 40/40 | Présence: 6/8 × 30 pts = 22.5/30 | GitHub: Dépôt trouvé (+5) | 2+ commit(s) (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 20/30 | Ajustement: 86.39% → 83.0% (-3.4 pts)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AZABAZE JIONGO ISMAEL</t>
+          <t>AZABAZE JIONGO ISMAEL BRICE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -976,29 +976,68 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>5/8</t>
+          <t>7/8</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>40</v>
       </c>
       <c r="G13" t="n">
-        <v>18.75</v>
+        <v>26.25</v>
       </c>
       <c r="H13" t="n">
         <v>25</v>
       </c>
       <c r="I13" t="n">
-        <v>79.48</v>
+        <v>85</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>79.48%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 5/8 × 30 pts = 18.75/30 | GitHub: Dépôt trouvé (+5) | 12+ commit(s) (+5) | 3+ commits (+5) | Actif &lt; 30j (+5) | R, documenté (+5) → 25/30 | Ajustement: 87.7% → 79.48% (-8.2 pts)</t>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 7/8 × 30 pts = 26.25/30 | GitHub ajusté: 25/30 | Ajustement: 95.55% → 85.0% (-10.5 pts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TARH-YENGUE YANNICK</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>3/8</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>55</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>55.0%</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Tests: 2 testé(s) × 20 pts = 40/40 | Présence: 3/8 × 30 pts = 11.25/30 | Aucun lien GitHub fourni. | Ajustement: 53.66% → 55.0% (+1.3 pts)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout des matricules depuis Google Sheets et correction des emails
</commit_message>
<xml_diff>
--- a/resultats_participation.xlsx
+++ b/resultats_participation.xlsx
@@ -417,8 +417,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -497,7 +497,11 @@
           <t>regispouho96@gmail.com</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cm-uds-22sci0176</t>
+        </is>
+      </c>
       <c r="D2" t="n">
         <v>2</v>
       </c>
@@ -540,7 +544,11 @@
           <t>pierredjibrilgamani@gmail.com</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CM-UDS23SCI0292</t>
+        </is>
+      </c>
       <c r="D3" t="n">
         <v>2</v>
       </c>
@@ -583,7 +591,11 @@
           <t>charonneyemeli@gmail.com</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CM- UDS- 23SCIO733</t>
+        </is>
+      </c>
       <c r="D4" t="n">
         <v>2</v>
       </c>
@@ -626,7 +638,11 @@
           <t>tsomejiobiko@gmail.com</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CM-UDS-25SCI0849</t>
+        </is>
+      </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
@@ -669,7 +685,11 @@
           <t>richellenoumedem2@gmail.com</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CM-UDS-25SCI0833</t>
+        </is>
+      </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
@@ -712,7 +732,11 @@
           <t>dupontdjeague@gmail.com</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CM-UDS-23SCI0483</t>
+        </is>
+      </c>
       <c r="D7" t="n">
         <v>5</v>
       </c>
@@ -755,7 +779,11 @@
           <t>dongmogirelle@gmail.com</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CM-UDS23SCI0763</t>
+        </is>
+      </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
@@ -798,7 +826,11 @@
           <t>arthurmbonde908@gmail.com</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CM-UDS-25SCI0763</t>
+        </is>
+      </c>
       <c r="D9" t="n">
         <v>2</v>
       </c>
@@ -841,7 +873,11 @@
           <t>sikatipierre@gmail.com</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CM-UDS-22SCI0756</t>
+        </is>
+      </c>
       <c r="D10" t="n">
         <v>5</v>
       </c>
@@ -884,7 +920,11 @@
           <t>dongmoivan242@gmail.com</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CM-UDS22SCI0440</t>
+        </is>
+      </c>
       <c r="D11" t="n">
         <v>2</v>
       </c>
@@ -927,7 +967,11 @@
           <t>andersontalisca237@gmail.com</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CM-UDS-23SCI1130</t>
+        </is>
+      </c>
       <c r="D12" t="n">
         <v>4</v>
       </c>
@@ -967,10 +1011,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ismaelbricejiongo@gmail.com</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>ismaeljiongo286@gmail.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CM-UDS-20SCI0186</t>
+        </is>
+      </c>
       <c r="D13" t="n">
         <v>2</v>
       </c>
@@ -1008,8 +1056,16 @@
           <t>TARH-YENGUE YANNICK</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>yannicktarhyengue235@gmail.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CM-UDS22SCI0923</t>
+        </is>
+      </c>
       <c r="D14" t="n">
         <v>2</v>
       </c>

</xml_diff>